<commit_message>
Fix double-space in 'Alcoholic beverages, tobacco' category name
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/cpi-national-by-category-monthly-en.xlsx
+++ b/data.mn/public/datasets/cpi-national-by-category-monthly-en.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -693,7 +693,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -903,7 +903,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -4443,7 +4443,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -4623,7 +4623,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C342" t="n">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C359" t="n">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C364" t="n">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C383" t="n">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C387" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C408" t="n">
@@ -6648,7 +6648,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C415" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C424" t="n">
@@ -6948,7 +6948,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C435" t="n">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C456" t="n">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C467" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C474" t="n">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C487" t="n">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C505" t="n">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C510" t="n">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C520" t="n">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C538" t="n">
@@ -8688,7 +8688,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C551" t="n">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C560" t="n">
@@ -9033,7 +9033,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C574" t="n">
@@ -9138,7 +9138,7 @@
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C581" t="n">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C593" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C609" t="n">
@@ -9633,7 +9633,7 @@
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C614" t="n">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C632" t="n">
@@ -10113,7 +10113,7 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C646" t="n">
@@ -10338,7 +10338,7 @@
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C661" t="n">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C673" t="n">
@@ -10668,7 +10668,7 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C683" t="n">
@@ -10713,7 +10713,7 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C686" t="n">
@@ -11028,7 +11028,7 @@
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C707" t="n">
@@ -11133,7 +11133,7 @@
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C714" t="n">
@@ -11418,7 +11418,7 @@
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C733" t="n">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C741" t="n">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C746" t="n">
@@ -11808,7 +11808,7 @@
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C759" t="n">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C771" t="n">
@@ -12288,7 +12288,7 @@
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C791" t="n">
@@ -12438,7 +12438,7 @@
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C801" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C816" t="n">
@@ -12783,7 +12783,7 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C824" t="n">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C840" t="n">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C843" t="n">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C859" t="n">
@@ -13563,7 +13563,7 @@
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C876" t="n">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C881" t="n">
@@ -13833,7 +13833,7 @@
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C894" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C902" t="n">
@@ -14283,7 +14283,7 @@
       </c>
       <c r="B924" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C924" t="n">
@@ -14403,7 +14403,7 @@
       </c>
       <c r="B932" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C932" t="n">
@@ -14508,7 +14508,7 @@
       </c>
       <c r="B939" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C939" t="n">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="B956" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C956" t="n">
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B963" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C963" t="n">
@@ -15108,7 +15108,7 @@
       </c>
       <c r="B979" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C979" t="n">
@@ -15378,7 +15378,7 @@
       </c>
       <c r="B997" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C997" t="n">
@@ -15468,7 +15468,7 @@
       </c>
       <c r="B1003" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1003" t="n">
@@ -15603,7 +15603,7 @@
       </c>
       <c r="B1012" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1012" t="n">
@@ -15873,7 +15873,7 @@
       </c>
       <c r="B1030" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1030" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B1044" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1044" t="n">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="B1049" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1049" t="n">
@@ -16383,7 +16383,7 @@
       </c>
       <c r="B1064" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1064" t="n">
@@ -16623,7 +16623,7 @@
       </c>
       <c r="B1080" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1080" t="n">
@@ -16713,7 +16713,7 @@
       </c>
       <c r="B1086" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1086" t="n">
@@ -16998,7 +16998,7 @@
       </c>
       <c r="B1105" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1105" t="n">
@@ -17148,7 +17148,7 @@
       </c>
       <c r="B1115" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1115" t="n">
@@ -17328,7 +17328,7 @@
       </c>
       <c r="B1127" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1127" t="n">
@@ -17463,7 +17463,7 @@
       </c>
       <c r="B1136" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1136" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B1149" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1149" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B1158" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1158" t="n">
@@ -18048,7 +18048,7 @@
       </c>
       <c r="B1175" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1175" t="n">
@@ -18183,7 +18183,7 @@
       </c>
       <c r="B1184" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1184" t="n">
@@ -18273,7 +18273,7 @@
       </c>
       <c r="B1190" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1190" t="n">
@@ -18618,7 +18618,7 @@
       </c>
       <c r="B1213" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1213" t="n">
@@ -18723,7 +18723,7 @@
       </c>
       <c r="B1220" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1220" t="n">
@@ -18963,7 +18963,7 @@
       </c>
       <c r="B1236" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1236" t="n">
@@ -19008,7 +19008,7 @@
       </c>
       <c r="B1239" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1239" t="n">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="B1255" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1255" t="n">
@@ -19473,7 +19473,7 @@
       </c>
       <c r="B1270" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1270" t="n">
@@ -19563,7 +19563,7 @@
       </c>
       <c r="B1276" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1276" t="n">
@@ -19758,7 +19758,7 @@
       </c>
       <c r="B1289" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1289" t="n">
@@ -20043,7 +20043,7 @@
       </c>
       <c r="B1308" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1308" t="n">
@@ -20178,7 +20178,7 @@
       </c>
       <c r="B1317" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1317" t="n">
@@ -20283,7 +20283,7 @@
       </c>
       <c r="B1324" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1324" t="n">
@@ -20493,7 +20493,7 @@
       </c>
       <c r="B1338" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1338" t="n">
@@ -20778,7 +20778,7 @@
       </c>
       <c r="B1357" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1357" t="n">
@@ -20793,7 +20793,7 @@
       </c>
       <c r="B1358" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1358" t="n">
@@ -21093,7 +21093,7 @@
       </c>
       <c r="B1378" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1378" t="n">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B1385" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1385" t="n">
@@ -21498,7 +21498,7 @@
       </c>
       <c r="B1405" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1405" t="n">
@@ -21618,7 +21618,7 @@
       </c>
       <c r="B1413" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1413" t="n">
@@ -21858,7 +21858,7 @@
       </c>
       <c r="B1429" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1429" t="n">
@@ -22038,7 +22038,7 @@
       </c>
       <c r="B1441" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1441" t="n">
@@ -22173,7 +22173,7 @@
       </c>
       <c r="B1450" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1450" t="n">
@@ -22398,7 +22398,7 @@
       </c>
       <c r="B1465" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1465" t="n">
@@ -22563,7 +22563,7 @@
       </c>
       <c r="B1476" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1476" t="n">
@@ -22638,7 +22638,7 @@
       </c>
       <c r="B1481" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1481" t="n">
@@ -22878,7 +22878,7 @@
       </c>
       <c r="B1497" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1497" t="n">
@@ -23208,7 +23208,7 @@
       </c>
       <c r="B1519" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1519" t="n">
@@ -23328,7 +23328,7 @@
       </c>
       <c r="B1527" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1527" t="n">
@@ -23568,7 +23568,7 @@
       </c>
       <c r="B1543" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1543" t="n">
@@ -23673,7 +23673,7 @@
       </c>
       <c r="B1550" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1550" t="n">
@@ -23808,7 +23808,7 @@
       </c>
       <c r="B1559" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1559" t="n">
@@ -24108,7 +24108,7 @@
       </c>
       <c r="B1579" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1579" t="n">
@@ -24348,7 +24348,7 @@
       </c>
       <c r="B1595" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1595" t="n">
@@ -24573,7 +24573,7 @@
       </c>
       <c r="B1610" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1610" t="n">
@@ -24708,7 +24708,7 @@
       </c>
       <c r="B1619" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1619" t="n">
@@ -24783,7 +24783,7 @@
       </c>
       <c r="B1624" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1624" t="n">
@@ -25038,7 +25038,7 @@
       </c>
       <c r="B1641" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1641" t="n">
@@ -25248,7 +25248,7 @@
       </c>
       <c r="B1655" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1655" t="n">
@@ -25503,7 +25503,7 @@
       </c>
       <c r="B1672" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1672" t="n">
@@ -25713,7 +25713,7 @@
       </c>
       <c r="B1686" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1686" t="n">
@@ -25863,7 +25863,7 @@
       </c>
       <c r="B1696" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1696" t="n">
@@ -26073,7 +26073,7 @@
       </c>
       <c r="B1710" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1710" t="n">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="B1727" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1727" t="n">
@@ -26433,7 +26433,7 @@
       </c>
       <c r="B1734" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1734" t="n">
@@ -26538,7 +26538,7 @@
       </c>
       <c r="B1741" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1741" t="n">
@@ -26898,7 +26898,7 @@
       </c>
       <c r="B1765" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1765" t="n">
@@ -27003,7 +27003,7 @@
       </c>
       <c r="B1772" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1772" t="n">
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B1784" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1784" t="n">
@@ -27438,7 +27438,7 @@
       </c>
       <c r="B1801" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1801" t="n">
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B1815" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1815" t="n">
@@ -27753,7 +27753,7 @@
       </c>
       <c r="B1822" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1822" t="n">
@@ -27978,7 +27978,7 @@
       </c>
       <c r="B1837" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1837" t="n">
@@ -28098,7 +28098,7 @@
       </c>
       <c r="B1845" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1845" t="n">
@@ -28443,7 +28443,7 @@
       </c>
       <c r="B1868" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1868" t="n">
@@ -28668,7 +28668,7 @@
       </c>
       <c r="B1883" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1883" t="n">
@@ -28743,7 +28743,7 @@
       </c>
       <c r="B1888" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1888" t="n">
@@ -29028,7 +29028,7 @@
       </c>
       <c r="B1907" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1907" t="n">
@@ -29208,7 +29208,7 @@
       </c>
       <c r="B1919" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1919" t="n">
@@ -29298,7 +29298,7 @@
       </c>
       <c r="B1925" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1925" t="n">
@@ -29583,7 +29583,7 @@
       </c>
       <c r="B1944" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1944" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B1956" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1956" t="n">
@@ -29973,7 +29973,7 @@
       </c>
       <c r="B1970" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1970" t="n">
@@ -30123,7 +30123,7 @@
       </c>
       <c r="B1980" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1980" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B1994" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C1994" t="n">
@@ -30438,7 +30438,7 @@
       </c>
       <c r="B2001" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2001" t="n">
@@ -30753,7 +30753,7 @@
       </c>
       <c r="B2022" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2022" t="n">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="B2036" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2036" t="n">
@@ -31128,7 +31128,7 @@
       </c>
       <c r="B2047" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2047" t="n">
@@ -31383,7 +31383,7 @@
       </c>
       <c r="B2064" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2064" t="n">
@@ -31533,7 +31533,7 @@
       </c>
       <c r="B2074" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2074" t="n">
@@ -31743,7 +31743,7 @@
       </c>
       <c r="B2088" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2088" t="n">
@@ -31848,7 +31848,7 @@
       </c>
       <c r="B2095" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2095" t="n">
@@ -32058,7 +32058,7 @@
       </c>
       <c r="B2109" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2109" t="n">
@@ -32193,7 +32193,7 @@
       </c>
       <c r="B2118" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2118" t="n">
@@ -32463,7 +32463,7 @@
       </c>
       <c r="B2136" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2136" t="n">
@@ -32598,7 +32598,7 @@
       </c>
       <c r="B2145" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2145" t="n">
@@ -32838,7 +32838,7 @@
       </c>
       <c r="B2161" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2161" t="n">
@@ -32973,7 +32973,7 @@
       </c>
       <c r="B2170" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2170" t="n">
@@ -33303,7 +33303,7 @@
       </c>
       <c r="B2192" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2192" t="n">
@@ -33483,7 +33483,7 @@
       </c>
       <c r="B2204" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2204" t="n">
@@ -33678,7 +33678,7 @@
       </c>
       <c r="B2217" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2217" t="n">
@@ -33888,7 +33888,7 @@
       </c>
       <c r="B2231" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2231" t="n">
@@ -34113,7 +34113,7 @@
       </c>
       <c r="B2246" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2246" t="n">
@@ -34278,7 +34278,7 @@
       </c>
       <c r="B2257" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2257" t="n">
@@ -34338,7 +34338,7 @@
       </c>
       <c r="B2261" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2261" t="n">
@@ -34653,7 +34653,7 @@
       </c>
       <c r="B2282" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2282" t="n">
@@ -34743,7 +34743,7 @@
       </c>
       <c r="B2288" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2288" t="n">
@@ -34953,7 +34953,7 @@
       </c>
       <c r="B2302" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2302" t="n">
@@ -35163,7 +35163,7 @@
       </c>
       <c r="B2316" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2316" t="n">
@@ -35418,7 +35418,7 @@
       </c>
       <c r="B2333" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2333" t="n">
@@ -35508,7 +35508,7 @@
       </c>
       <c r="B2339" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2339" t="n">
@@ -35838,7 +35838,7 @@
       </c>
       <c r="B2361" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2361" t="n">
@@ -36063,7 +36063,7 @@
       </c>
       <c r="B2376" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2376" t="n">
@@ -36153,7 +36153,7 @@
       </c>
       <c r="B2382" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2382" t="n">
@@ -36303,7 +36303,7 @@
       </c>
       <c r="B2392" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2392" t="n">
@@ -36648,7 +36648,7 @@
       </c>
       <c r="B2415" t="inlineStr">
         <is>
-          <t>Alcoholic  beverages, tobacco</t>
+          <t>Alcoholic beverages, tobacco</t>
         </is>
       </c>
       <c r="C2415" t="n">

</xml_diff>